<commit_message>
feat(export): enhance skula excel generation with dynamic row management
Implement dynamic row insertion and removal in the SKULA export service
to handle varying numbers of transport, lodging, and other expenses.
This ensures the Excel template structure remains intact regardless of
the expense count.

- Add dynamic row manipulation logic to `TravelOrderExportService`
- Implement company branding and styling in the exported XML
- Add support for merged cells and hidden columns in SKULA format
- Update `TravelOrderExportTest` to validate dynamic row positioning
  and new XML structure requirements
</commit_message>
<xml_diff>
--- a/SKULA_Adnan_Mandzo_latest_fixed.xlsx
+++ b/SKULA_Adnan_Mandzo_latest_fixed.xlsx
@@ -1297,15 +1297,32 @@
     <col min="3" max="3" width="24.140625" style="3" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" style="3" customWidth="1"/>
     <col min="5" max="5" width="34.42578125" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="9.140625" style="1"/>
+    <col min="7" max="16384" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25" ht="54" customHeight="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="8"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">qla.dev
+Braće Mulić 81, Sarajevo
+Bosnia</t>
+          </r>
+        </is>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OBRAČUN TROŠKOVA SLUŽBENOG PUTOVANJA</t>
+        </is>
+      </c>
       <c r="D1" s="74"/>
       <c r="E1" s="74"/>
     </row>
@@ -1459,7 +1476,14 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERVAUTO BELG-LUX S.A. TOTALENERGIES WAARLOOS ANTWERPEN</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">SERVAUTO BELG-LUX S.A. TOTALENERGIES WAARLOOS ANTWERPEN</t>
+          </r>
         </is>
       </c>
       <c r="C14" s="91">
@@ -1478,7 +1502,14 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          </r>
         </is>
       </c>
       <c r="C15" s="91">
@@ -1497,7 +1528,14 @@
       </c>
       <c r="B16" s="93" t="inlineStr">
         <is>
-          <t xml:space="preserve">ART HOTEL ROTTERDAM</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">ART HOTEL ROTTERDAM</t>
+          </r>
         </is>
       </c>
       <c r="C16" s="91">
@@ -1516,7 +1554,14 @@
       </c>
       <c r="B17" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          </r>
         </is>
       </c>
       <c r="C17" s="91">
@@ -1563,7 +1608,14 @@
       </c>
       <c r="B20" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          </r>
         </is>
       </c>
       <c r="C20" s="91">
@@ -1582,7 +1634,14 @@
       </c>
       <c r="B21" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHELL STAT. SANDELINGEN-OOST</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">SHELL STAT. SANDELINGEN-OOST</t>
+          </r>
         </is>
       </c>
       <c r="C21" s="91">
@@ -1601,7 +1660,14 @@
       </c>
       <c r="B22" s="45" t="inlineStr">
         <is>
-          <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">GEMEENTE ROTTERDAM</t>
+          </r>
         </is>
       </c>
       <c r="C22" s="91">
@@ -1624,7 +1690,6 @@
       <c r="E23" s="90">
         <v>245.32</v>
       </c>
-      <c r="F23" s="20"/>
     </row>
     <row r="24" spans="1:6" s="3" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
@@ -1649,7 +1714,14 @@
       </c>
       <c r="B25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOOKING.COM</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">BOOKING.COM</t>
+          </r>
         </is>
       </c>
       <c r="C25" s="91">
@@ -1668,7 +1740,14 @@
       </c>
       <c r="B26" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOTALENERGIES DAMPREMY</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">TOTALENERGIES DAMPREMY</t>
+          </r>
         </is>
       </c>
       <c r="C26" s="91">
@@ -1687,7 +1766,14 @@
       </c>
       <c r="B27" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">GATE BAR 21</t>
+          <r>
+            <rPr>
+              <sz val="9"/>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">GATE BAR 21</t>
+          </r>
         </is>
       </c>
       <c r="C27" s="91">
@@ -1867,8 +1953,9 @@
       <c r="A48" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:E1"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A38:D38"/>
   </mergeCells>

</xml_diff>